<commit_message>
Add Gr12 science priority overrides, re-run engine v2.5: 54 clashes
39 Grade 12 students' science courses (543, 546, 530, 531) are now
treated as graduation_required via student_priority_overrides.json.
All 39 overrides successfully seated. Clashes reduced from 69 to 54,
placement rate improved from 98.9% to 99.1%.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Teacher_Schedule_Review_and_Tally.xlsx
+++ b/Teacher_Schedule_Review_and_Tally.xlsx
@@ -7498,14 +7498,14 @@
         </is>
       </c>
       <c r="C255" s="2" t="n"/>
-      <c r="D255" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E255" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D255" s="6" t="inlineStr">
+        <is>
+          <t>131-3: British Literature H - 3</t>
+        </is>
+      </c>
+      <c r="E255" s="6" t="inlineStr">
+        <is>
+          <t>131-3: British Literature H - 3</t>
         </is>
       </c>
       <c r="F255" s="2" t="n"/>
@@ -7668,14 +7668,14 @@
         </is>
       </c>
       <c r="C260" s="2" t="n"/>
-      <c r="D260" s="6" t="inlineStr">
-        <is>
-          <t>131-3: British Literature H - 3</t>
-        </is>
-      </c>
-      <c r="E260" s="6" t="inlineStr">
-        <is>
-          <t>131-3: British Literature H - 3</t>
+      <c r="D260" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E260" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F260" s="2" t="n"/>
@@ -7752,11 +7752,11 @@
         </is>
       </c>
       <c r="C263" s="2" t="n"/>
-      <c r="D263" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E263" s="7" t="n">
-        <v>3</v>
+      <c r="D263" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E263" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F263" s="2" t="n"/>
       <c r="G263" s="7" t="n">
@@ -9815,14 +9815,14 @@
         </is>
       </c>
       <c r="C339" s="2" t="n"/>
-      <c r="D339" s="6" t="inlineStr">
-        <is>
-          <t>543-1: Anatomy/Physiology H - 1</t>
-        </is>
-      </c>
-      <c r="E339" s="6" t="inlineStr">
-        <is>
-          <t>543-1: Anatomy/Physiology H - 1</t>
+      <c r="D339" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E339" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F339" s="2" t="n"/>
@@ -9985,14 +9985,14 @@
         </is>
       </c>
       <c r="C344" s="2" t="n"/>
-      <c r="D344" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E344" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D344" s="6" t="inlineStr">
+        <is>
+          <t>542-1: Anatomy/Physiology - 1</t>
+        </is>
+      </c>
+      <c r="E344" s="6" t="inlineStr">
+        <is>
+          <t>542-1: Anatomy/Physiology - 1</t>
         </is>
       </c>
       <c r="F344" s="2" t="n"/>
@@ -10021,12 +10021,12 @@
       <c r="C345" s="2" t="n"/>
       <c r="D345" s="6" t="inlineStr">
         <is>
-          <t>542-1: Anatomy/Physiology - 1</t>
+          <t>543-1: Anatomy/Physiology H - 1</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
         <is>
-          <t>542-1: Anatomy/Physiology - 1</t>
+          <t>543-1: Anatomy/Physiology H - 1</t>
         </is>
       </c>
       <c r="F345" s="2" t="n"/>
@@ -10248,14 +10248,14 @@
         </is>
       </c>
       <c r="C354" s="2" t="n"/>
-      <c r="D354" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E354" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D354" s="6" t="inlineStr">
+        <is>
+          <t>430-4: Algebra II/Trig - 4</t>
+        </is>
+      </c>
+      <c r="E354" s="6" t="inlineStr">
+        <is>
+          <t>430-4: Algebra II/Trig - 4</t>
         </is>
       </c>
       <c r="F354" s="2" t="n"/>
@@ -10316,14 +10316,14 @@
         </is>
       </c>
       <c r="C356" s="2" t="n"/>
-      <c r="D356" s="6" t="inlineStr">
-        <is>
-          <t>430-4: Algebra II/Trig - 4</t>
-        </is>
-      </c>
-      <c r="E356" s="6" t="inlineStr">
-        <is>
-          <t>430-4: Algebra II/Trig - 4</t>
+      <c r="D356" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E356" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F356" s="2" t="n"/>
@@ -10401,10 +10401,10 @@
       </c>
       <c r="C359" s="2" t="n"/>
       <c r="D359" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E359" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F359" s="2" t="n"/>
       <c r="G359" s="7" t="n">
@@ -13461,9 +13461,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E471" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E471" s="6" t="inlineStr">
+        <is>
+          <t>765-2-S: AP Macroeconomics - 2</t>
         </is>
       </c>
       <c r="F471" s="2" t="n"/>
@@ -13665,9 +13665,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E477" s="6" t="inlineStr">
-        <is>
-          <t>765-2-S: AP Macroeconomics - 2</t>
+      <c r="E477" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F477" s="2" t="n"/>
@@ -13889,14 +13889,14 @@
         </is>
       </c>
       <c r="C486" s="2" t="n"/>
-      <c r="D486" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E486" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D486" s="6" t="inlineStr">
+        <is>
+          <t>530-2: Physics - 2</t>
+        </is>
+      </c>
+      <c r="E486" s="6" t="inlineStr">
+        <is>
+          <t>530-2: Physics - 2</t>
         </is>
       </c>
       <c r="F486" s="2" t="n"/>
@@ -13957,14 +13957,14 @@
         </is>
       </c>
       <c r="C488" s="2" t="n"/>
-      <c r="D488" s="6" t="inlineStr">
-        <is>
-          <t>530-2: Physics - 2</t>
-        </is>
-      </c>
-      <c r="E488" s="6" t="inlineStr">
-        <is>
-          <t>530-2: Physics - 2</t>
+      <c r="D488" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E488" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F488" s="2" t="n"/>
@@ -14041,11 +14041,11 @@
         </is>
       </c>
       <c r="C491" s="2" t="n"/>
-      <c r="D491" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E491" s="7" t="n">
-        <v>3</v>
+      <c r="D491" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E491" s="9" t="n">
+        <v>5</v>
       </c>
       <c r="F491" s="2" t="n"/>
       <c r="G491" s="9" t="n">
@@ -14587,12 +14587,12 @@
       <c r="C511" s="2" t="n"/>
       <c r="D511" s="6" t="inlineStr">
         <is>
-          <t>830-4: Theology 11 - 4; 851-1-F: Spirituality of Vocation - 1</t>
+          <t>851-1-F: Spirituality of Vocation - 1</t>
         </is>
       </c>
       <c r="E511" s="6" t="inlineStr">
         <is>
-          <t>830-4: Theology 11 - 4; 851-8-S: Spirituality of Vocation - 8</t>
+          <t>851-8-S: Spirituality of Vocation - 8</t>
         </is>
       </c>
       <c r="F511" s="2" t="n"/>
@@ -14619,14 +14619,14 @@
         </is>
       </c>
       <c r="C512" s="2" t="n"/>
-      <c r="D512" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D512" s="6" t="inlineStr">
+        <is>
+          <t>830-4: Theology 11 - 4</t>
         </is>
       </c>
       <c r="E512" s="6" t="inlineStr">
         <is>
-          <t>851-5-S: Spirituality of Vocation - 5</t>
+          <t>830-4: Theology 11 - 4; 851-5-S: Spirituality of Vocation - 5</t>
         </is>
       </c>
       <c r="F512" s="2" t="n"/>
@@ -14704,7 +14704,7 @@
       </c>
       <c r="C515" s="2" t="n"/>
       <c r="D515" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E515" s="7" t="n">
         <v>3</v>
@@ -15111,9 +15111,9 @@
         </is>
       </c>
       <c r="C531" s="2" t="n"/>
-      <c r="D531" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D531" s="6" t="inlineStr">
+        <is>
+          <t>220-1-F: Music Theory - 1</t>
         </is>
       </c>
       <c r="E531" s="7" t="inlineStr">
@@ -15145,9 +15145,9 @@
         </is>
       </c>
       <c r="C532" s="2" t="n"/>
-      <c r="D532" s="6" t="inlineStr">
-        <is>
-          <t>220-1-F: Music Theory - 1</t>
+      <c r="D532" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E532" s="7" t="inlineStr">
@@ -19416,12 +19416,12 @@
       <c r="C687" s="2" t="n"/>
       <c r="D687" s="6" t="inlineStr">
         <is>
-          <t>830-8: Theology 11 - 8</t>
+          <t>830-9: Theology 11 - 9</t>
         </is>
       </c>
       <c r="E687" s="6" t="inlineStr">
         <is>
-          <t>830-8: Theology 11 - 8</t>
+          <t>830-9: Theology 11 - 9</t>
         </is>
       </c>
       <c r="F687" s="2" t="n"/>
@@ -19484,12 +19484,12 @@
       <c r="C689" s="2" t="n"/>
       <c r="D689" s="6" t="inlineStr">
         <is>
-          <t>830-7: Theology 11 - 7</t>
+          <t>830-8: Theology 11 - 8</t>
         </is>
       </c>
       <c r="E689" s="6" t="inlineStr">
         <is>
-          <t>830-7: Theology 11 - 7</t>
+          <t>830-8: Theology 11 - 8</t>
         </is>
       </c>
       <c r="F689" s="2" t="n"/>
@@ -19518,12 +19518,12 @@
       <c r="C690" s="2" t="n"/>
       <c r="D690" s="6" t="inlineStr">
         <is>
-          <t>830-6: Theology 11 - 6</t>
+          <t>830-7: Theology 11 - 7</t>
         </is>
       </c>
       <c r="E690" s="6" t="inlineStr">
         <is>
-          <t>830-6: Theology 11 - 6</t>
+          <t>830-7: Theology 11 - 7</t>
         </is>
       </c>
       <c r="F690" s="2" t="n"/>
@@ -19550,14 +19550,14 @@
         </is>
       </c>
       <c r="C691" s="2" t="n"/>
-      <c r="D691" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E691" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D691" s="6" t="inlineStr">
+        <is>
+          <t>830-6: Theology 11 - 6</t>
+        </is>
+      </c>
+      <c r="E691" s="6" t="inlineStr">
+        <is>
+          <t>830-6: Theology 11 - 6</t>
         </is>
       </c>
       <c r="F691" s="2" t="n"/>
@@ -19584,14 +19584,14 @@
         </is>
       </c>
       <c r="C692" s="2" t="n"/>
-      <c r="D692" s="6" t="inlineStr">
-        <is>
-          <t>830-9: Theology 11 - 9</t>
-        </is>
-      </c>
-      <c r="E692" s="6" t="inlineStr">
-        <is>
-          <t>830-9: Theology 11 - 9</t>
+      <c r="D692" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E692" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F692" s="2" t="n"/>
@@ -19669,10 +19669,10 @@
       </c>
       <c r="C695" s="2" t="n"/>
       <c r="D695" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E695" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F695" s="2" t="n"/>
       <c r="G695" s="7" t="n">
@@ -20110,14 +20110,14 @@
         </is>
       </c>
       <c r="C712" s="2" t="n"/>
-      <c r="D712" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E712" s="6" t="inlineStr">
-        <is>
-          <t>2024-2-S: TV/Film Process and Principles - 2</t>
+      <c r="D712" s="6" t="inlineStr">
+        <is>
+          <t>2034-1-F: TV/Film Production &amp; Editing I - 1</t>
+        </is>
+      </c>
+      <c r="E712" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F712" s="2" t="n"/>
@@ -20178,9 +20178,9 @@
         </is>
       </c>
       <c r="C714" s="2" t="n"/>
-      <c r="D714" s="6" t="inlineStr">
-        <is>
-          <t>2034-1-F: TV/Film Production &amp; Editing I - 1</t>
+      <c r="D714" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E714" s="6" t="inlineStr">
@@ -20217,9 +20217,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E715" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E715" s="6" t="inlineStr">
+        <is>
+          <t>2024-2-S: TV/Film Process and Principles - 2</t>
         </is>
       </c>
       <c r="F715" s="2" t="n"/>
@@ -20331,10 +20331,10 @@
       </c>
       <c r="C719" s="2" t="n"/>
       <c r="D719" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E719" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E719" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F719" s="2" t="n"/>
       <c r="G719" s="7" t="n">
@@ -22427,14 +22427,14 @@
         </is>
       </c>
       <c r="C796" s="2" t="n"/>
-      <c r="D796" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E796" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D796" s="6" t="inlineStr">
+        <is>
+          <t>531-2: Physics H - 2</t>
+        </is>
+      </c>
+      <c r="E796" s="6" t="inlineStr">
+        <is>
+          <t>531-2: Physics H - 2</t>
         </is>
       </c>
       <c r="F796" s="2" t="n"/>
@@ -22597,14 +22597,14 @@
         </is>
       </c>
       <c r="C801" s="2" t="n"/>
-      <c r="D801" s="6" t="inlineStr">
-        <is>
-          <t>531-2: Physics H - 2</t>
-        </is>
-      </c>
-      <c r="E801" s="6" t="inlineStr">
-        <is>
-          <t>531-2: Physics H - 2</t>
+      <c r="D801" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E801" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F801" s="2" t="n"/>
@@ -24379,14 +24379,14 @@
         </is>
       </c>
       <c r="C867" s="2" t="n"/>
-      <c r="D867" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E867" s="6" t="inlineStr">
-        <is>
-          <t>732-2-S: Business Law - 2</t>
+      <c r="D867" s="6" t="inlineStr">
+        <is>
+          <t>732-3-F: Business Law - 3</t>
+        </is>
+      </c>
+      <c r="E867" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F867" s="2" t="n"/>
@@ -24413,9 +24413,9 @@
         </is>
       </c>
       <c r="C868" s="2" t="n"/>
-      <c r="D868" s="6" t="inlineStr">
-        <is>
-          <t>732-3-F: Business Law - 3</t>
+      <c r="D868" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E868" s="7" t="inlineStr">
@@ -24452,9 +24452,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E869" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E869" s="6" t="inlineStr">
+        <is>
+          <t>732-2-S: Business Law - 2</t>
         </is>
       </c>
       <c r="F869" s="2" t="n"/>
@@ -24637,7 +24637,7 @@
         <v>4</v>
       </c>
       <c r="E875" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F875" s="2" t="n"/>
       <c r="G875" s="7" t="n">

</xml_diff>

<commit_message>
Add 6th section of 310 (Period F, Tuesta), hard cap enforcement at 28
- Added 6th section of 310 Spanish I in Period F for Tuesta (Template 6 Sheet 2)
- Updated Template 7: 310 sections 5→6, max enrollment 28; 520 max enrollment 28
- Updated priority_assignments.json: 310 sections 5→6
- Implemented HARD_CAP_ENFORCEMENT in engine at all 6 placement points:
  Phase B greedy, CSP resolve, full_reseat() greedy, full_reseat_fast() greedy,
  and post-bump recovery in both full_reseat() and full_reseat_fast()
- Engine v2.5 re-run: 55 clashes, 99.1% placement, 100% grad req fulfillment
- 310 enrollments now balanced: 28/12/13/12/28/28 across periods A/B/C/D/E/G
- 520 enrollments all under cap: 22/22/9/19/22 across periods A/B/C/F/G
- Regenerated all 3 reports: Master Section Report, Teacher Schedule Review, Remaining Clashes

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Teacher_Schedule_Review_and_Tally.xlsx
+++ b/Teacher_Schedule_Review_and_Tally.xlsx
@@ -1939,14 +1939,14 @@
         </is>
       </c>
       <c r="C53" s="2" t="n"/>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>610-3-F: Health/PE - 3</t>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>610-10-S: Health/PE - 10</t>
+          <t>610-4-S: Health/PE - 4</t>
         </is>
       </c>
       <c r="F53" s="2" t="n"/>
@@ -1973,14 +1973,14 @@
         </is>
       </c>
       <c r="C54" s="2" t="n"/>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>610-3-F: Health/PE - 3</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>610-4-S: Health/PE - 4</t>
+          <t>610-10-S: Health/PE - 10</t>
         </is>
       </c>
       <c r="F54" s="2" t="n"/>
@@ -2007,14 +2007,14 @@
         </is>
       </c>
       <c r="C55" s="2" t="n"/>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>610-6-S: Health/PE - 6</t>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>610-5-F: Health/PE - 5</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F55" s="2" t="n"/>
@@ -2075,14 +2075,14 @@
         </is>
       </c>
       <c r="C57" s="2" t="n"/>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>610-5-F: Health/PE - 5</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>610-6-S: Health/PE - 6</t>
         </is>
       </c>
       <c r="F57" s="2" t="n"/>
@@ -2129,7 +2129,7 @@
         <v>3</v>
       </c>
       <c r="E59" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="7" t="n">
@@ -2533,14 +2533,14 @@
         </is>
       </c>
       <c r="C75" s="2" t="n"/>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>491-1: AP Computer Science Principles - 1</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>472-2-S: Web Design - 2</t>
+          <t>491-1: AP Computer Science Principles - 1</t>
         </is>
       </c>
       <c r="F75" s="2" t="n"/>
@@ -2603,12 +2603,12 @@
       <c r="C77" s="2" t="n"/>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>491-1: AP Computer Science Principles - 1</t>
+          <t>496-1: AP Cybersecurity - 1</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>491-1: AP Computer Science Principles - 1</t>
+          <t>496-1: AP Cybersecurity - 1</t>
         </is>
       </c>
       <c r="F77" s="2" t="n"/>
@@ -2669,14 +2669,14 @@
         </is>
       </c>
       <c r="C79" s="2" t="n"/>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>494-1-F: Applied Programming - 1; 473-1-F: Introduction to Programming - 1</t>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>473-2-S: Introduction to Programming - 2</t>
+          <t>472-2-S: Web Design - 2</t>
         </is>
       </c>
       <c r="F79" s="2" t="n"/>
@@ -2703,14 +2703,14 @@
         </is>
       </c>
       <c r="C80" s="2" t="n"/>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>494-1-F: Applied Programming - 1; 473-1-F: Introduction to Programming - 1</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>473-2-S: Introduction to Programming - 2</t>
         </is>
       </c>
       <c r="F80" s="2" t="n"/>
@@ -2737,14 +2737,14 @@
         </is>
       </c>
       <c r="C81" s="2" t="n"/>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>496-1: AP Cybersecurity - 1</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="inlineStr">
-        <is>
-          <t>496-1: AP Cybersecurity - 1</t>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F81" s="2" t="n"/>
@@ -3528,12 +3528,12 @@
       <c r="C111" s="2" t="n"/>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>642-3-F: Nutrition &amp; Fitness/PE - 3</t>
+          <t>631-3-F: CPR-AED Training/PE - 3</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>631-2-S: CPR-AED Training/PE - 2</t>
+          <t>642-2-S: Nutrition &amp; Fitness/PE - 2</t>
         </is>
       </c>
       <c r="F111" s="2" t="n"/>
@@ -3562,12 +3562,12 @@
       <c r="C112" s="2" t="n"/>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>631-1-F: CPR-AED Training/PE - 1</t>
-        </is>
-      </c>
-      <c r="E112" s="6" t="inlineStr">
-        <is>
-          <t>642-2-S: Nutrition &amp; Fitness/PE - 2</t>
+          <t>642-3-F: Nutrition &amp; Fitness/PE - 3</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F112" s="2" t="n"/>
@@ -3698,7 +3698,7 @@
       <c r="C116" s="2" t="n"/>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>631-3-F: CPR-AED Training/PE - 3</t>
+          <t>631-1-F: CPR-AED Training/PE - 1</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
@@ -3735,9 +3735,9 @@
           <t>642-1-F: Nutrition &amp; Fitness/PE - 1</t>
         </is>
       </c>
-      <c r="E117" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t>631-2-S: CPR-AED Training/PE - 2</t>
         </is>
       </c>
       <c r="F117" s="2" t="n"/>
@@ -3783,8 +3783,8 @@
       <c r="D119" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E119" s="9" t="n">
-        <v>4</v>
+      <c r="E119" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="F119" s="2" t="n"/>
       <c r="G119" s="7" t="n">
@@ -4029,12 +4029,12 @@
       <c r="C128" s="2" t="n"/>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>546-1: Forensics - 1</t>
+          <t>546-2: Forensics - 2</t>
         </is>
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>546-1: Forensics - 1</t>
+          <t>546-2: Forensics - 2</t>
         </is>
       </c>
       <c r="F128" s="2" t="n"/>
@@ -4063,12 +4063,12 @@
       <c r="C129" s="2" t="n"/>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>546-2: Forensics - 2</t>
+          <t>546-1: Forensics - 1</t>
         </is>
       </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>546-2: Forensics - 2</t>
+          <t>546-1: Forensics - 1</t>
         </is>
       </c>
       <c r="F129" s="2" t="n"/>
@@ -4188,14 +4188,14 @@
         </is>
       </c>
       <c r="C135" s="2" t="n"/>
-      <c r="D135" s="6" t="inlineStr">
-        <is>
-          <t>727-3-F: Sports and Entertainment Marketing - 3</t>
-        </is>
-      </c>
-      <c r="E135" s="6" t="inlineStr">
-        <is>
-          <t>758-2-S: Bloomberg Market Concepts - 2</t>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F135" s="2" t="n"/>
@@ -4324,9 +4324,9 @@
         </is>
       </c>
       <c r="C139" s="2" t="n"/>
-      <c r="D139" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>727-3-F: Sports and Entertainment Marketing - 3</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
@@ -4360,12 +4360,12 @@
       <c r="C140" s="2" t="n"/>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>732-1-F: Business Law - 1; 757-3: International Business Strategies - 3</t>
+          <t>757-3: International Business Strategies - 3</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
         <is>
-          <t>757-3: International Business Strategies - 3</t>
+          <t>758-2-S: Bloomberg Market Concepts - 2; 757-3: International Business Strategies - 3</t>
         </is>
       </c>
       <c r="F140" s="2" t="n"/>
@@ -4392,9 +4392,9 @@
         </is>
       </c>
       <c r="C141" s="2" t="n"/>
-      <c r="D141" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>732-1-F: Business Law - 1</t>
         </is>
       </c>
       <c r="E141" s="6" t="inlineStr">
@@ -4443,7 +4443,7 @@
       </c>
       <c r="C143" s="2" t="n"/>
       <c r="D143" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E143" s="7" t="n">
         <v>3</v>
@@ -4553,14 +4553,14 @@
         </is>
       </c>
       <c r="C148" s="2" t="n"/>
-      <c r="D148" s="6" t="inlineStr">
-        <is>
-          <t>620-3-F: Driver's Ed/PE - 3</t>
-        </is>
-      </c>
-      <c r="E148" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D148" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E148" s="6" t="inlineStr">
+        <is>
+          <t>620-4-S: Driver's Ed/PE - 4</t>
         </is>
       </c>
       <c r="F148" s="2" t="n"/>
@@ -4689,14 +4689,14 @@
         </is>
       </c>
       <c r="C152" s="2" t="n"/>
-      <c r="D152" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E152" s="6" t="inlineStr">
-        <is>
-          <t>620-4-S: Driver's Ed/PE - 4</t>
+      <c r="D152" s="6" t="inlineStr">
+        <is>
+          <t>620-3-F: Driver's Ed/PE - 3</t>
+        </is>
+      </c>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F152" s="2" t="n"/>
@@ -4774,10 +4774,10 @@
       </c>
       <c r="C155" s="2" t="n"/>
       <c r="D155" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E155" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F155" s="2" t="n"/>
       <c r="G155" s="9" t="n">
@@ -4954,12 +4954,12 @@
       <c r="C162" s="2" t="n"/>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>440-2: Precalculus - 2</t>
+          <t>440-3: Precalculus - 3</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr">
         <is>
-          <t>440-2: Precalculus - 2</t>
+          <t>440-3: Precalculus - 3</t>
         </is>
       </c>
       <c r="F162" s="2" t="n"/>
@@ -4988,12 +4988,12 @@
       <c r="C163" s="2" t="n"/>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>440-3: Precalculus - 3</t>
+          <t>440-2: Precalculus - 2</t>
         </is>
       </c>
       <c r="E163" s="6" t="inlineStr">
         <is>
-          <t>440-3: Precalculus - 3</t>
+          <t>440-2: Precalculus - 2</t>
         </is>
       </c>
       <c r="F163" s="2" t="n"/>
@@ -5285,12 +5285,12 @@
       <c r="C174" s="2" t="n"/>
       <c r="D174" s="6" t="inlineStr">
         <is>
-          <t>111-2: Composition &amp; Literature H - 2</t>
+          <t>111-1: Composition &amp; Literature H - 1</t>
         </is>
       </c>
       <c r="E174" s="6" t="inlineStr">
         <is>
-          <t>111-2: Composition &amp; Literature H - 2</t>
+          <t>111-1: Composition &amp; Literature H - 1</t>
         </is>
       </c>
       <c r="F174" s="2" t="n"/>
@@ -5353,12 +5353,12 @@
       <c r="C176" s="2" t="n"/>
       <c r="D176" s="6" t="inlineStr">
         <is>
-          <t>111-1: Composition &amp; Literature H - 1</t>
+          <t>111-2: Composition &amp; Literature H - 2</t>
         </is>
       </c>
       <c r="E176" s="6" t="inlineStr">
         <is>
-          <t>111-1: Composition &amp; Literature H - 1</t>
+          <t>111-2: Composition &amp; Literature H - 2</t>
         </is>
       </c>
       <c r="F176" s="2" t="n"/>
@@ -5546,9 +5546,9 @@
         </is>
       </c>
       <c r="C184" s="2" t="n"/>
-      <c r="D184" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>241-1-F: Studio Art I - 1</t>
         </is>
       </c>
       <c r="E184" s="6" t="inlineStr">
@@ -5614,14 +5614,14 @@
         </is>
       </c>
       <c r="C186" s="2" t="n"/>
-      <c r="D186" s="6" t="inlineStr">
-        <is>
-          <t>242-1-F: Studio Art II - 1; 243-1-F: Studio Art III - 1</t>
-        </is>
-      </c>
-      <c r="E186" s="6" t="inlineStr">
-        <is>
-          <t>242-2-S: Studio Art II - 2; 243-2-S: Studio Art III - 2</t>
+      <c r="D186" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F186" s="2" t="n"/>
@@ -5650,12 +5650,12 @@
       <c r="C187" s="2" t="n"/>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>241-1-F: Studio Art I - 1</t>
+          <t>242-1-F: Studio Art II - 1; 243-1-F: Studio Art III - 1</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>249-2-S: Adv Painting - 2</t>
+          <t>242-2-S: Studio Art II - 2; 243-2-S: Studio Art III - 2</t>
         </is>
       </c>
       <c r="F187" s="2" t="n"/>
@@ -5721,9 +5721,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E189" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>249-2-S: Adv Painting - 2</t>
         </is>
       </c>
       <c r="F189" s="2" t="n"/>
@@ -5845,12 +5845,12 @@
       <c r="C195" s="2" t="n"/>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>520-5: Chemistry - 5</t>
+          <t>520-4: Chemistry - 4</t>
         </is>
       </c>
       <c r="E195" s="6" t="inlineStr">
         <is>
-          <t>520-5: Chemistry - 5</t>
+          <t>520-4: Chemistry - 4</t>
         </is>
       </c>
       <c r="F195" s="2" t="n"/>
@@ -5879,12 +5879,12 @@
       <c r="C196" s="2" t="n"/>
       <c r="D196" s="6" t="inlineStr">
         <is>
-          <t>520-4: Chemistry - 4</t>
+          <t>520-5: Chemistry - 5</t>
         </is>
       </c>
       <c r="E196" s="6" t="inlineStr">
         <is>
-          <t>520-4: Chemistry - 4</t>
+          <t>520-5: Chemistry - 5</t>
         </is>
       </c>
       <c r="F196" s="2" t="n"/>
@@ -5913,12 +5913,12 @@
       <c r="C197" s="2" t="n"/>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>520-3: Chemistry - 3</t>
+          <t>520-2: Chemistry - 2</t>
         </is>
       </c>
       <c r="E197" s="6" t="inlineStr">
         <is>
-          <t>520-3: Chemistry - 3</t>
+          <t>520-2: Chemistry - 2</t>
         </is>
       </c>
       <c r="F197" s="2" t="n"/>
@@ -6015,12 +6015,12 @@
       <c r="C200" s="2" t="n"/>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t>520-2: Chemistry - 2</t>
+          <t>520-3: Chemistry - 3</t>
         </is>
       </c>
       <c r="E200" s="6" t="inlineStr">
         <is>
-          <t>520-2: Chemistry - 2</t>
+          <t>520-3: Chemistry - 3</t>
         </is>
       </c>
       <c r="F200" s="2" t="n"/>
@@ -6208,14 +6208,14 @@
         </is>
       </c>
       <c r="C208" s="2" t="n"/>
-      <c r="D208" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E208" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t>130-2: British Literature - 2</t>
+        </is>
+      </c>
+      <c r="E208" s="6" t="inlineStr">
+        <is>
+          <t>130-2: British Literature - 2</t>
         </is>
       </c>
       <c r="F208" s="2" t="n"/>
@@ -6378,14 +6378,14 @@
         </is>
       </c>
       <c r="C213" s="2" t="n"/>
-      <c r="D213" s="6" t="inlineStr">
-        <is>
-          <t>130-2: British Literature - 2</t>
-        </is>
-      </c>
-      <c r="E213" s="6" t="inlineStr">
-        <is>
-          <t>130-2: British Literature - 2</t>
+      <c r="D213" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E213" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F213" s="2" t="n"/>
@@ -6507,12 +6507,12 @@
       <c r="C219" s="2" t="n"/>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>726-1-F: Business Concepts - 1</t>
-        </is>
-      </c>
-      <c r="E219" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+          <t>729-2: AP Business with Personal Finance - 2</t>
+        </is>
+      </c>
+      <c r="E219" s="6" t="inlineStr">
+        <is>
+          <t>729-2: AP Business with Personal Finance - 2</t>
         </is>
       </c>
       <c r="F219" s="2" t="n"/>
@@ -6609,7 +6609,7 @@
       <c r="C222" s="2" t="n"/>
       <c r="D222" s="6" t="inlineStr">
         <is>
-          <t>726-3-F: Business Concepts - 3</t>
+          <t>726-1-F: Business Concepts - 1</t>
         </is>
       </c>
       <c r="E222" s="6" t="inlineStr">
@@ -6675,9 +6675,9 @@
         </is>
       </c>
       <c r="C224" s="2" t="n"/>
-      <c r="D224" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D224" s="6" t="inlineStr">
+        <is>
+          <t>726-3-F: Business Concepts - 3</t>
         </is>
       </c>
       <c r="E224" s="7" t="inlineStr">
@@ -6709,14 +6709,14 @@
         </is>
       </c>
       <c r="C225" s="2" t="n"/>
-      <c r="D225" s="6" t="inlineStr">
-        <is>
-          <t>729-2: AP Business with Personal Finance - 2</t>
-        </is>
-      </c>
-      <c r="E225" s="6" t="inlineStr">
-        <is>
-          <t>729-2: AP Business with Personal Finance - 2</t>
+      <c r="D225" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E225" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F225" s="2" t="n"/>
@@ -6760,10 +6760,10 @@
       </c>
       <c r="C227" s="2" t="n"/>
       <c r="D227" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E227" s="9" t="n">
         <v>5</v>
-      </c>
-      <c r="E227" s="9" t="n">
-        <v>4</v>
       </c>
       <c r="F227" s="2" t="n"/>
       <c r="G227" s="9" t="n">
@@ -6938,9 +6938,9 @@
         </is>
       </c>
       <c r="C234" s="2" t="n"/>
-      <c r="D234" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D234" s="6" t="inlineStr">
+        <is>
+          <t>228-1-F: Adv Theater Production - 1; 227-1-F: Intermediate Theater - 1</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -7040,9 +7040,9 @@
         </is>
       </c>
       <c r="C237" s="2" t="n"/>
-      <c r="D237" s="6" t="inlineStr">
-        <is>
-          <t>228-1-F: Adv Theater Production - 1; 227-1-F: Intermediate Theater - 1</t>
+      <c r="D237" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="C239" s="2" t="n"/>
       <c r="D239" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E239" s="7" t="n">
         <v>1</v>
@@ -8822,14 +8822,14 @@
         </is>
       </c>
       <c r="C303" s="2" t="n"/>
-      <c r="D303" s="6" t="inlineStr">
-        <is>
-          <t>120-5: American Literature - 5</t>
-        </is>
-      </c>
-      <c r="E303" s="6" t="inlineStr">
-        <is>
-          <t>120-5: American Literature - 5</t>
+      <c r="D303" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E303" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F303" s="2" t="n"/>
@@ -8856,14 +8856,14 @@
         </is>
       </c>
       <c r="C304" s="2" t="n"/>
-      <c r="D304" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E304" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D304" s="6" t="inlineStr">
+        <is>
+          <t>120-5: American Literature - 5</t>
+        </is>
+      </c>
+      <c r="E304" s="6" t="inlineStr">
+        <is>
+          <t>120-5: American Literature - 5</t>
         </is>
       </c>
       <c r="F304" s="2" t="n"/>
@@ -8892,12 +8892,12 @@
       <c r="C305" s="2" t="n"/>
       <c r="D305" s="6" t="inlineStr">
         <is>
-          <t>120-2: American Literature - 2</t>
+          <t>120-3: American Literature - 3</t>
         </is>
       </c>
       <c r="E305" s="6" t="inlineStr">
         <is>
-          <t>120-2: American Literature - 2</t>
+          <t>120-3: American Literature - 3</t>
         </is>
       </c>
       <c r="F305" s="2" t="n"/>
@@ -8960,12 +8960,12 @@
       <c r="C307" s="2" t="n"/>
       <c r="D307" s="6" t="inlineStr">
         <is>
-          <t>120-3: American Literature - 3</t>
+          <t>120-1: American Literature - 1</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
         <is>
-          <t>120-3: American Literature - 3</t>
+          <t>120-1: American Literature - 1</t>
         </is>
       </c>
       <c r="F307" s="2" t="n"/>
@@ -8994,12 +8994,12 @@
       <c r="C308" s="2" t="n"/>
       <c r="D308" s="6" t="inlineStr">
         <is>
-          <t>120-1: American Literature - 1</t>
+          <t>120-2: American Literature - 2</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
         <is>
-          <t>120-1: American Literature - 1</t>
+          <t>120-2: American Literature - 2</t>
         </is>
       </c>
       <c r="F308" s="2" t="n"/>
@@ -9077,10 +9077,10 @@
       </c>
       <c r="C311" s="2" t="n"/>
       <c r="D311" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E311" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F311" s="2" t="n"/>
       <c r="G311" s="7" t="n">
@@ -9554,12 +9554,12 @@
       <c r="C329" s="2" t="n"/>
       <c r="D329" s="6" t="inlineStr">
         <is>
-          <t>810-2: Theology 9 - 2</t>
+          <t>820-2: Theology 10 - 2</t>
         </is>
       </c>
       <c r="E329" s="6" t="inlineStr">
         <is>
-          <t>810-2: Theology 9 - 2</t>
+          <t>820-2: Theology 10 - 2</t>
         </is>
       </c>
       <c r="F329" s="2" t="n"/>
@@ -9588,12 +9588,12 @@
       <c r="C330" s="2" t="n"/>
       <c r="D330" s="6" t="inlineStr">
         <is>
-          <t>820-1: Theology 10 - 1</t>
+          <t>810-1: Theology 9 - 1</t>
         </is>
       </c>
       <c r="E330" s="6" t="inlineStr">
         <is>
-          <t>820-1: Theology 10 - 1</t>
+          <t>810-1: Theology 9 - 1</t>
         </is>
       </c>
       <c r="F330" s="2" t="n"/>
@@ -9622,12 +9622,12 @@
       <c r="C331" s="2" t="n"/>
       <c r="D331" s="6" t="inlineStr">
         <is>
-          <t>820-2: Theology 10 - 2</t>
+          <t>810-3: Theology 9 - 3</t>
         </is>
       </c>
       <c r="E331" s="6" t="inlineStr">
         <is>
-          <t>820-2: Theology 10 - 2</t>
+          <t>810-3: Theology 9 - 3</t>
         </is>
       </c>
       <c r="F331" s="2" t="n"/>
@@ -9656,12 +9656,12 @@
       <c r="C332" s="2" t="n"/>
       <c r="D332" s="6" t="inlineStr">
         <is>
-          <t>810-3: Theology 9 - 3</t>
+          <t>820-1: Theology 10 - 1</t>
         </is>
       </c>
       <c r="E332" s="6" t="inlineStr">
         <is>
-          <t>810-3: Theology 9 - 3</t>
+          <t>820-1: Theology 10 - 1</t>
         </is>
       </c>
       <c r="F332" s="2" t="n"/>
@@ -9690,12 +9690,12 @@
       <c r="C333" s="2" t="n"/>
       <c r="D333" s="6" t="inlineStr">
         <is>
-          <t>810-1: Theology 9 - 1</t>
+          <t>810-2: Theology 9 - 2</t>
         </is>
       </c>
       <c r="E333" s="6" t="inlineStr">
         <is>
-          <t>810-1: Theology 9 - 1</t>
+          <t>810-2: Theology 9 - 2</t>
         </is>
       </c>
       <c r="F333" s="2" t="n"/>
@@ -11209,12 +11209,12 @@
       <c r="C389" s="2" t="n"/>
       <c r="D389" s="6" t="inlineStr">
         <is>
-          <t>420-1: Geometry - 1</t>
+          <t>412-1: Algebra I - 1</t>
         </is>
       </c>
       <c r="E389" s="6" t="inlineStr">
         <is>
-          <t>420-1: Geometry - 1</t>
+          <t>412-1: Algebra I - 1</t>
         </is>
       </c>
       <c r="F389" s="2" t="n"/>
@@ -11243,12 +11243,12 @@
       <c r="C390" s="2" t="n"/>
       <c r="D390" s="6" t="inlineStr">
         <is>
-          <t>412-1: Algebra I - 1</t>
+          <t>420-1: Geometry - 1</t>
         </is>
       </c>
       <c r="E390" s="6" t="inlineStr">
         <is>
-          <t>412-1: Algebra I - 1</t>
+          <t>420-1: Geometry - 1</t>
         </is>
       </c>
       <c r="F390" s="2" t="n"/>
@@ -12499,12 +12499,12 @@
       <c r="C436" s="2" t="n"/>
       <c r="D436" s="6" t="inlineStr">
         <is>
-          <t>810-4: Theology 9 - 4</t>
+          <t>810-7: Theology 9 - 7</t>
         </is>
       </c>
       <c r="E436" s="6" t="inlineStr">
         <is>
-          <t>810-4: Theology 9 - 4</t>
+          <t>810-7: Theology 9 - 7</t>
         </is>
       </c>
       <c r="F436" s="2" t="n"/>
@@ -12531,14 +12531,14 @@
         </is>
       </c>
       <c r="C437" s="2" t="n"/>
-      <c r="D437" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E437" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D437" s="6" t="inlineStr">
+        <is>
+          <t>810-4: Theology 9 - 4</t>
+        </is>
+      </c>
+      <c r="E437" s="6" t="inlineStr">
+        <is>
+          <t>810-4: Theology 9 - 4</t>
         </is>
       </c>
       <c r="F437" s="2" t="n"/>
@@ -12567,12 +12567,12 @@
       <c r="C438" s="2" t="n"/>
       <c r="D438" s="6" t="inlineStr">
         <is>
-          <t>810-6: Theology 9 - 6</t>
+          <t>810-8: Theology 9 - 8</t>
         </is>
       </c>
       <c r="E438" s="6" t="inlineStr">
         <is>
-          <t>810-6: Theology 9 - 6</t>
+          <t>810-8: Theology 9 - 8</t>
         </is>
       </c>
       <c r="F438" s="2" t="n"/>
@@ -12599,14 +12599,14 @@
         </is>
       </c>
       <c r="C439" s="2" t="n"/>
-      <c r="D439" s="6" t="inlineStr">
-        <is>
-          <t>810-7: Theology 9 - 7</t>
-        </is>
-      </c>
-      <c r="E439" s="6" t="inlineStr">
-        <is>
-          <t>810-7: Theology 9 - 7</t>
+      <c r="D439" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E439" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F439" s="2" t="n"/>
@@ -12633,14 +12633,14 @@
         </is>
       </c>
       <c r="C440" s="2" t="n"/>
-      <c r="D440" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E440" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D440" s="6" t="inlineStr">
+        <is>
+          <t>810-6: Theology 9 - 6</t>
+        </is>
+      </c>
+      <c r="E440" s="6" t="inlineStr">
+        <is>
+          <t>810-6: Theology 9 - 6</t>
         </is>
       </c>
       <c r="F440" s="2" t="n"/>
@@ -12667,14 +12667,14 @@
         </is>
       </c>
       <c r="C441" s="2" t="n"/>
-      <c r="D441" s="6" t="inlineStr">
-        <is>
-          <t>810-8: Theology 9 - 8</t>
-        </is>
-      </c>
-      <c r="E441" s="6" t="inlineStr">
-        <is>
-          <t>810-8: Theology 9 - 8</t>
+      <c r="D441" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E441" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F441" s="2" t="n"/>
@@ -12717,11 +12717,11 @@
         </is>
       </c>
       <c r="C443" s="2" t="n"/>
-      <c r="D443" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E443" s="7" t="n">
-        <v>2</v>
+      <c r="D443" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E443" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F443" s="2" t="n"/>
       <c r="G443" s="7" t="n">
@@ -13456,9 +13456,9 @@
         </is>
       </c>
       <c r="C471" s="2" t="n"/>
-      <c r="D471" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D471" s="6" t="inlineStr">
+        <is>
+          <t>766-2-F: AP Microeconomics - 2</t>
         </is>
       </c>
       <c r="E471" s="6" t="inlineStr">
@@ -13490,9 +13490,9 @@
         </is>
       </c>
       <c r="C472" s="2" t="n"/>
-      <c r="D472" s="6" t="inlineStr">
-        <is>
-          <t>766-2-F: AP Microeconomics - 2</t>
+      <c r="D472" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E472" s="7" t="inlineStr">
@@ -13792,9 +13792,9 @@
           <t>UNASSIGNED</t>
         </is>
       </c>
-      <c r="E483" s="6" t="inlineStr">
-        <is>
-          <t>595-2-S: Engineering Design - 2</t>
+      <c r="E483" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F483" s="2" t="n"/>
@@ -13857,12 +13857,12 @@
       <c r="C485" s="2" t="n"/>
       <c r="D485" s="6" t="inlineStr">
         <is>
-          <t>530-3: Physics - 3</t>
+          <t>530-2: Physics - 2</t>
         </is>
       </c>
       <c r="E485" s="6" t="inlineStr">
         <is>
-          <t>530-3: Physics - 3</t>
+          <t>530-2: Physics - 2</t>
         </is>
       </c>
       <c r="F485" s="2" t="n"/>
@@ -13891,12 +13891,12 @@
       <c r="C486" s="2" t="n"/>
       <c r="D486" s="6" t="inlineStr">
         <is>
-          <t>530-2: Physics - 2</t>
+          <t>530-3: Physics - 3</t>
         </is>
       </c>
       <c r="E486" s="6" t="inlineStr">
         <is>
-          <t>530-2: Physics - 2</t>
+          <t>530-3: Physics - 3</t>
         </is>
       </c>
       <c r="F486" s="2" t="n"/>
@@ -13996,9 +13996,9 @@
           <t>595-1-F: Engineering Design - 1</t>
         </is>
       </c>
-      <c r="E489" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E489" s="6" t="inlineStr">
+        <is>
+          <t>595-2-S: Engineering Design - 2</t>
         </is>
       </c>
       <c r="F489" s="2" t="n"/>
@@ -14045,7 +14045,7 @@
         <v>4</v>
       </c>
       <c r="E491" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F491" s="2" t="n"/>
       <c r="G491" s="9" t="n">
@@ -14186,14 +14186,14 @@
         </is>
       </c>
       <c r="C497" s="2" t="n"/>
-      <c r="D497" s="6" t="inlineStr">
-        <is>
-          <t>820-3: Theology 10 - 3</t>
-        </is>
-      </c>
-      <c r="E497" s="6" t="inlineStr">
-        <is>
-          <t>820-3: Theology 10 - 3</t>
+      <c r="D497" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E497" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F497" s="2" t="n"/>
@@ -14220,14 +14220,14 @@
         </is>
       </c>
       <c r="C498" s="2" t="n"/>
-      <c r="D498" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E498" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D498" s="6" t="inlineStr">
+        <is>
+          <t>820-5: Theology 10 - 5</t>
+        </is>
+      </c>
+      <c r="E498" s="6" t="inlineStr">
+        <is>
+          <t>820-5: Theology 10 - 5</t>
         </is>
       </c>
       <c r="F498" s="2" t="n"/>
@@ -14254,14 +14254,14 @@
         </is>
       </c>
       <c r="C499" s="2" t="n"/>
-      <c r="D499" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E499" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D499" s="6" t="inlineStr">
+        <is>
+          <t>820-3: Theology 10 - 3</t>
+        </is>
+      </c>
+      <c r="E499" s="6" t="inlineStr">
+        <is>
+          <t>820-3: Theology 10 - 3</t>
         </is>
       </c>
       <c r="F499" s="2" t="n"/>
@@ -14322,14 +14322,14 @@
         </is>
       </c>
       <c r="C501" s="2" t="n"/>
-      <c r="D501" s="6" t="inlineStr">
-        <is>
-          <t>820-5: Theology 10 - 5</t>
-        </is>
-      </c>
-      <c r="E501" s="6" t="inlineStr">
-        <is>
-          <t>820-5: Theology 10 - 5</t>
+      <c r="D501" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E501" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F501" s="2" t="n"/>
@@ -14519,12 +14519,12 @@
       <c r="C509" s="2" t="n"/>
       <c r="D509" s="6" t="inlineStr">
         <is>
-          <t>851-3-F: Spirituality of Vocation - 3</t>
-        </is>
-      </c>
-      <c r="E509" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+          <t>851-1-F: Spirituality of Vocation - 1</t>
+        </is>
+      </c>
+      <c r="E509" s="6" t="inlineStr">
+        <is>
+          <t>851-8-S: Spirituality of Vocation - 8</t>
         </is>
       </c>
       <c r="F509" s="2" t="n"/>
@@ -14551,14 +14551,14 @@
         </is>
       </c>
       <c r="C510" s="2" t="n"/>
-      <c r="D510" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E510" s="6" t="inlineStr">
-        <is>
-          <t>851-6-S: Spirituality of Vocation - 6</t>
+      <c r="D510" s="6" t="inlineStr">
+        <is>
+          <t>851-3-F: Spirituality of Vocation - 3</t>
+        </is>
+      </c>
+      <c r="E510" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F510" s="2" t="n"/>
@@ -14585,14 +14585,14 @@
         </is>
       </c>
       <c r="C511" s="2" t="n"/>
-      <c r="D511" s="6" t="inlineStr">
-        <is>
-          <t>851-1-F: Spirituality of Vocation - 1</t>
+      <c r="D511" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E511" s="6" t="inlineStr">
         <is>
-          <t>851-8-S: Spirituality of Vocation - 8</t>
+          <t>851-5-S: Spirituality of Vocation - 5</t>
         </is>
       </c>
       <c r="F511" s="2" t="n"/>
@@ -14621,12 +14621,12 @@
       <c r="C512" s="2" t="n"/>
       <c r="D512" s="6" t="inlineStr">
         <is>
+          <t>830-4: Theology 11 - 4; 851-2-F: Spirituality of Vocation - 2</t>
+        </is>
+      </c>
+      <c r="E512" s="6" t="inlineStr">
+        <is>
           <t>830-4: Theology 11 - 4</t>
-        </is>
-      </c>
-      <c r="E512" s="6" t="inlineStr">
-        <is>
-          <t>830-4: Theology 11 - 4; 851-5-S: Spirituality of Vocation - 5</t>
         </is>
       </c>
       <c r="F512" s="2" t="n"/>
@@ -14653,14 +14653,14 @@
         </is>
       </c>
       <c r="C513" s="2" t="n"/>
-      <c r="D513" s="6" t="inlineStr">
-        <is>
-          <t>851-2-F: Spirituality of Vocation - 2</t>
-        </is>
-      </c>
-      <c r="E513" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D513" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E513" s="6" t="inlineStr">
+        <is>
+          <t>851-6-S: Spirituality of Vocation - 6</t>
         </is>
       </c>
       <c r="F513" s="2" t="n"/>
@@ -14704,7 +14704,7 @@
       </c>
       <c r="C515" s="2" t="n"/>
       <c r="D515" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E515" s="7" t="n">
         <v>3</v>
@@ -14782,12 +14782,12 @@
       <c r="C519" s="2" t="n"/>
       <c r="D519" s="6" t="inlineStr">
         <is>
-          <t>820-9: Theology 10 - 9</t>
+          <t>820-7: Theology 10 - 7</t>
         </is>
       </c>
       <c r="E519" s="6" t="inlineStr">
         <is>
-          <t>820-9: Theology 10 - 9</t>
+          <t>820-7: Theology 10 - 7</t>
         </is>
       </c>
       <c r="F519" s="2" t="n"/>
@@ -14882,14 +14882,14 @@
         </is>
       </c>
       <c r="C522" s="2" t="n"/>
-      <c r="D522" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E522" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D522" s="6" t="inlineStr">
+        <is>
+          <t>820-9: Theology 10 - 9</t>
+        </is>
+      </c>
+      <c r="E522" s="6" t="inlineStr">
+        <is>
+          <t>820-9: Theology 10 - 9</t>
         </is>
       </c>
       <c r="F522" s="2" t="n"/>
@@ -14950,14 +14950,14 @@
         </is>
       </c>
       <c r="C524" s="2" t="n"/>
-      <c r="D524" s="6" t="inlineStr">
-        <is>
-          <t>820-7: Theology 10 - 7</t>
-        </is>
-      </c>
-      <c r="E524" s="6" t="inlineStr">
-        <is>
-          <t>820-7: Theology 10 - 7</t>
+      <c r="D524" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E524" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F524" s="2" t="n"/>
@@ -15034,11 +15034,11 @@
         </is>
       </c>
       <c r="C527" s="2" t="n"/>
-      <c r="D527" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E527" s="7" t="n">
-        <v>3</v>
+      <c r="D527" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E527" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F527" s="2" t="n"/>
       <c r="G527" s="7" t="n">
@@ -15283,12 +15283,12 @@
       <c r="C536" s="2" t="n"/>
       <c r="D536" s="6" t="inlineStr">
         <is>
-          <t>203-1: Guitar Ensemble - 1; 203-2: Guitar Ensemble - 2; 201-1-F: Introduction to Guitar - 1; 201-3-F: Introduction to Guitar - 3</t>
+          <t>209-1: String Orchestra - 1</t>
         </is>
       </c>
       <c r="E536" s="6" t="inlineStr">
         <is>
-          <t>203-1: Guitar Ensemble - 1; 203-2: Guitar Ensemble - 2; 201-2-S: Introduction to Guitar - 2</t>
+          <t>209-1: String Orchestra - 1</t>
         </is>
       </c>
       <c r="F536" s="2" t="n"/>
@@ -15317,12 +15317,12 @@
       <c r="C537" s="2" t="n"/>
       <c r="D537" s="6" t="inlineStr">
         <is>
-          <t>209-1: String Orchestra - 1</t>
+          <t>203-1: Guitar Ensemble - 1; 203-2: Guitar Ensemble - 2; 201-1-F: Introduction to Guitar - 1; 201-3-F: Introduction to Guitar - 3</t>
         </is>
       </c>
       <c r="E537" s="6" t="inlineStr">
         <is>
-          <t>209-1: String Orchestra - 1</t>
+          <t>203-1: Guitar Ensemble - 1; 203-2: Guitar Ensemble - 2; 201-2-S: Introduction to Guitar - 2</t>
         </is>
       </c>
       <c r="F537" s="2" t="n"/>
@@ -15442,14 +15442,14 @@
         </is>
       </c>
       <c r="C543" s="2" t="n"/>
-      <c r="D543" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E543" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D543" s="6" t="inlineStr">
+        <is>
+          <t>763-2: AP U.S. Government &amp; Politics - 2</t>
+        </is>
+      </c>
+      <c r="E543" s="6" t="inlineStr">
+        <is>
+          <t>763-2: AP U.S. Government &amp; Politics - 2</t>
         </is>
       </c>
       <c r="F543" s="2" t="n"/>
@@ -15646,14 +15646,14 @@
         </is>
       </c>
       <c r="C549" s="2" t="n"/>
-      <c r="D549" s="6" t="inlineStr">
-        <is>
-          <t>763-2: AP U.S. Government &amp; Politics - 2</t>
-        </is>
-      </c>
-      <c r="E549" s="6" t="inlineStr">
-        <is>
-          <t>763-2: AP U.S. Government &amp; Politics - 2</t>
+      <c r="D549" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E549" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F549" s="2" t="n"/>
@@ -15945,12 +15945,12 @@
       <c r="C560" s="2" t="n"/>
       <c r="D560" s="6" t="inlineStr">
         <is>
-          <t>955-6: Academic Support - 6</t>
+          <t>955-7: Academic Support - 7</t>
         </is>
       </c>
       <c r="E560" s="6" t="inlineStr">
         <is>
-          <t>955-6: Academic Support - 6</t>
+          <t>955-7: Academic Support - 7</t>
         </is>
       </c>
       <c r="F560" s="2" t="n"/>
@@ -15979,12 +15979,12 @@
       <c r="C561" s="2" t="n"/>
       <c r="D561" s="6" t="inlineStr">
         <is>
-          <t>955-7: Academic Support - 7</t>
+          <t>955-6: Academic Support - 6</t>
         </is>
       </c>
       <c r="E561" s="6" t="inlineStr">
         <is>
-          <t>955-7: Academic Support - 7</t>
+          <t>955-6: Academic Support - 6</t>
         </is>
       </c>
       <c r="F561" s="2" t="n"/>
@@ -16174,12 +16174,12 @@
       <c r="C569" s="2" t="n"/>
       <c r="D569" s="6" t="inlineStr">
         <is>
-          <t>580-3-F: Robotics Engineering - 3</t>
-        </is>
-      </c>
-      <c r="E569" s="6" t="inlineStr">
-        <is>
-          <t>570-2-S: Introduction to Robotics - 2</t>
+          <t>580-1-F: Robotics Engineering - 1</t>
+        </is>
+      </c>
+      <c r="E569" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F569" s="2" t="n"/>
@@ -16208,12 +16208,12 @@
       <c r="C570" s="2" t="n"/>
       <c r="D570" s="6" t="inlineStr">
         <is>
-          <t>580-1-F: Robotics Engineering - 1</t>
-        </is>
-      </c>
-      <c r="E570" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+          <t>580-3-F: Robotics Engineering - 3</t>
+        </is>
+      </c>
+      <c r="E570" s="6" t="inlineStr">
+        <is>
+          <t>570-2-S: Introduction to Robotics - 2</t>
         </is>
       </c>
       <c r="F570" s="2" t="n"/>
@@ -16361,8 +16361,8 @@
       <c r="D575" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E575" s="7" t="n">
-        <v>3</v>
+      <c r="E575" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F575" s="2" t="n"/>
       <c r="G575" s="7" t="n">
@@ -16435,14 +16435,14 @@
         </is>
       </c>
       <c r="C579" s="2" t="n"/>
-      <c r="D579" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E579" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D579" s="6" t="inlineStr">
+        <is>
+          <t>521-4: Chemistry H - 4</t>
+        </is>
+      </c>
+      <c r="E579" s="6" t="inlineStr">
+        <is>
+          <t>521-4: Chemistry H - 4</t>
         </is>
       </c>
       <c r="F579" s="2" t="n"/>
@@ -16537,14 +16537,14 @@
         </is>
       </c>
       <c r="C582" s="2" t="n"/>
-      <c r="D582" s="6" t="inlineStr">
-        <is>
-          <t>521-4: Chemistry H - 4</t>
-        </is>
-      </c>
-      <c r="E582" s="6" t="inlineStr">
-        <is>
-          <t>521-4: Chemistry H - 4</t>
+      <c r="D582" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E582" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F582" s="2" t="n"/>
@@ -16573,12 +16573,12 @@
       <c r="C583" s="2" t="n"/>
       <c r="D583" s="6" t="inlineStr">
         <is>
-          <t>521-3: Chemistry H - 3</t>
+          <t>521-1: Chemistry H - 1</t>
         </is>
       </c>
       <c r="E583" s="6" t="inlineStr">
         <is>
-          <t>521-3: Chemistry H - 3</t>
+          <t>521-1: Chemistry H - 1</t>
         </is>
       </c>
       <c r="F583" s="2" t="n"/>
@@ -16641,12 +16641,12 @@
       <c r="C585" s="2" t="n"/>
       <c r="D585" s="6" t="inlineStr">
         <is>
-          <t>521-1: Chemistry H - 1</t>
+          <t>521-3: Chemistry H - 3</t>
         </is>
       </c>
       <c r="E585" s="6" t="inlineStr">
         <is>
-          <t>521-1: Chemistry H - 1</t>
+          <t>521-3: Chemistry H - 3</t>
         </is>
       </c>
       <c r="F585" s="2" t="n"/>
@@ -16689,11 +16689,11 @@
         </is>
       </c>
       <c r="C587" s="2" t="n"/>
-      <c r="D587" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="E587" s="9" t="n">
-        <v>5</v>
+      <c r="D587" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E587" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F587" s="2" t="n"/>
       <c r="G587" s="9" t="n">
@@ -16836,12 +16836,12 @@
       <c r="C593" s="2" t="n"/>
       <c r="D593" s="6" t="inlineStr">
         <is>
-          <t>720-2: U.S. History I - 2</t>
+          <t>720-1: U.S. History I - 1</t>
         </is>
       </c>
       <c r="E593" s="6" t="inlineStr">
         <is>
-          <t>720-2: U.S. History I - 2</t>
+          <t>720-1: U.S. History I - 1</t>
         </is>
       </c>
       <c r="F593" s="2" t="n"/>
@@ -16870,12 +16870,12 @@
       <c r="C594" s="2" t="n"/>
       <c r="D594" s="6" t="inlineStr">
         <is>
-          <t>720-1: U.S. History I - 1</t>
+          <t>720-2: U.S. History I - 2</t>
         </is>
       </c>
       <c r="E594" s="6" t="inlineStr">
         <is>
-          <t>720-1: U.S. History I - 1</t>
+          <t>720-2: U.S. History I - 2</t>
         </is>
       </c>
       <c r="F594" s="2" t="n"/>
@@ -17863,12 +17863,12 @@
       <c r="C630" s="2" t="n"/>
       <c r="D630" s="6" t="inlineStr">
         <is>
-          <t>352-1: AP Italian - 1</t>
+          <t>332-1: Italian III - 1</t>
         </is>
       </c>
       <c r="E630" s="6" t="inlineStr">
         <is>
-          <t>352-1: AP Italian - 1</t>
+          <t>332-1: Italian III - 1</t>
         </is>
       </c>
       <c r="F630" s="2" t="n"/>
@@ -17897,12 +17897,12 @@
       <c r="C631" s="2" t="n"/>
       <c r="D631" s="6" t="inlineStr">
         <is>
-          <t>332-1: Italian III - 1</t>
+          <t>352-1: AP Italian - 1</t>
         </is>
       </c>
       <c r="E631" s="6" t="inlineStr">
         <is>
-          <t>332-1: Italian III - 1</t>
+          <t>352-1: AP Italian - 1</t>
         </is>
       </c>
       <c r="F631" s="2" t="n"/>
@@ -18754,12 +18754,12 @@
       <c r="C663" s="2" t="n"/>
       <c r="D663" s="6" t="inlineStr">
         <is>
-          <t>149-2: AP English Literature - 2</t>
+          <t>149-1: AP English Literature - 1</t>
         </is>
       </c>
       <c r="E663" s="6" t="inlineStr">
         <is>
-          <t>149-2: AP English Literature - 2</t>
+          <t>149-1: AP English Literature - 1</t>
         </is>
       </c>
       <c r="F663" s="2" t="n"/>
@@ -18820,14 +18820,14 @@
         </is>
       </c>
       <c r="C665" s="2" t="n"/>
-      <c r="D665" s="6" t="inlineStr">
-        <is>
-          <t>110-1: Composition &amp; Literature - 1</t>
-        </is>
-      </c>
-      <c r="E665" s="6" t="inlineStr">
-        <is>
-          <t>110-1: Composition &amp; Literature - 1</t>
+      <c r="D665" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E665" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F665" s="2" t="n"/>
@@ -18888,14 +18888,14 @@
         </is>
       </c>
       <c r="C667" s="2" t="n"/>
-      <c r="D667" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E667" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D667" s="6" t="inlineStr">
+        <is>
+          <t>110-1: Composition &amp; Literature - 1</t>
+        </is>
+      </c>
+      <c r="E667" s="6" t="inlineStr">
+        <is>
+          <t>110-1: Composition &amp; Literature - 1</t>
         </is>
       </c>
       <c r="F667" s="2" t="n"/>
@@ -18958,12 +18958,12 @@
       <c r="C669" s="2" t="n"/>
       <c r="D669" s="6" t="inlineStr">
         <is>
-          <t>149-1: AP English Literature - 1</t>
+          <t>149-2: AP English Literature - 2</t>
         </is>
       </c>
       <c r="E669" s="6" t="inlineStr">
         <is>
-          <t>149-1: AP English Literature - 1</t>
+          <t>149-2: AP English Literature - 2</t>
         </is>
       </c>
       <c r="F669" s="2" t="n"/>
@@ -19006,11 +19006,11 @@
         </is>
       </c>
       <c r="C671" s="2" t="n"/>
-      <c r="D671" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E671" s="7" t="n">
-        <v>2</v>
+      <c r="D671" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E671" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F671" s="2" t="n"/>
       <c r="G671" s="9" t="n">
@@ -19119,12 +19119,12 @@
       <c r="C676" s="2" t="n"/>
       <c r="D676" s="6" t="inlineStr">
         <is>
-          <t>410-2: Algebra I - 2</t>
+          <t>410-1: Algebra I - 1</t>
         </is>
       </c>
       <c r="E676" s="6" t="inlineStr">
         <is>
-          <t>410-2: Algebra I - 2</t>
+          <t>410-1: Algebra I - 1</t>
         </is>
       </c>
       <c r="F676" s="2" t="n"/>
@@ -19153,12 +19153,12 @@
       <c r="C677" s="2" t="n"/>
       <c r="D677" s="6" t="inlineStr">
         <is>
-          <t>410-1: Algebra I - 1</t>
+          <t>420-3: Geometry - 3</t>
         </is>
       </c>
       <c r="E677" s="6" t="inlineStr">
         <is>
-          <t>410-1: Algebra I - 1</t>
+          <t>420-3: Geometry - 3</t>
         </is>
       </c>
       <c r="F677" s="2" t="n"/>
@@ -19187,12 +19187,12 @@
       <c r="C678" s="2" t="n"/>
       <c r="D678" s="6" t="inlineStr">
         <is>
-          <t>420-3: Geometry - 3</t>
+          <t>410-3: Algebra I - 3</t>
         </is>
       </c>
       <c r="E678" s="6" t="inlineStr">
         <is>
-          <t>420-3: Geometry - 3</t>
+          <t>410-3: Algebra I - 3</t>
         </is>
       </c>
       <c r="F678" s="2" t="n"/>
@@ -19219,14 +19219,14 @@
         </is>
       </c>
       <c r="C679" s="2" t="n"/>
-      <c r="D679" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E679" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D679" s="6" t="inlineStr">
+        <is>
+          <t>410-2: Algebra I - 2</t>
+        </is>
+      </c>
+      <c r="E679" s="6" t="inlineStr">
+        <is>
+          <t>410-2: Algebra I - 2</t>
         </is>
       </c>
       <c r="F679" s="2" t="n"/>
@@ -19287,14 +19287,14 @@
         </is>
       </c>
       <c r="C681" s="2" t="n"/>
-      <c r="D681" s="6" t="inlineStr">
-        <is>
-          <t>410-3: Algebra I - 3</t>
-        </is>
-      </c>
-      <c r="E681" s="6" t="inlineStr">
-        <is>
-          <t>410-3: Algebra I - 3</t>
+      <c r="D681" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E681" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F681" s="2" t="n"/>
@@ -19338,10 +19338,10 @@
       </c>
       <c r="C683" s="2" t="n"/>
       <c r="D683" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E683" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F683" s="2" t="n"/>
       <c r="G683" s="7" t="n">
@@ -20081,9 +20081,9 @@
           <t>2024-1-F: TV/Film Process and Principles - 1</t>
         </is>
       </c>
-      <c r="E711" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="E711" s="6" t="inlineStr">
+        <is>
+          <t>2044-2-S: TV/Film Production II - 2</t>
         </is>
       </c>
       <c r="F711" s="2" t="n"/>
@@ -20178,14 +20178,14 @@
         </is>
       </c>
       <c r="C714" s="2" t="n"/>
-      <c r="D714" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E714" s="6" t="inlineStr">
-        <is>
-          <t>2054-2-S: Digital Media - 2</t>
+      <c r="D714" s="6" t="inlineStr">
+        <is>
+          <t>2054-1-F: Digital Media - 1</t>
+        </is>
+      </c>
+      <c r="E714" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F714" s="2" t="n"/>
@@ -20253,7 +20253,7 @@
       </c>
       <c r="E716" s="6" t="inlineStr">
         <is>
-          <t>2044-2-S: TV/Film Production II - 2</t>
+          <t>2054-2-S: Digital Media - 2</t>
         </is>
       </c>
       <c r="F716" s="2" t="n"/>
@@ -20280,9 +20280,9 @@
         </is>
       </c>
       <c r="C717" s="2" t="n"/>
-      <c r="D717" s="6" t="inlineStr">
-        <is>
-          <t>2054-1-F: Digital Media - 1</t>
+      <c r="D717" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E717" s="6" t="inlineStr">
@@ -20330,11 +20330,11 @@
         </is>
       </c>
       <c r="C719" s="2" t="n"/>
-      <c r="D719" s="7" t="n">
+      <c r="D719" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E719" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="E719" s="9" t="n">
-        <v>4</v>
       </c>
       <c r="F719" s="2" t="n"/>
       <c r="G719" s="7" t="n">
@@ -20409,12 +20409,12 @@
       <c r="C723" s="2" t="n"/>
       <c r="D723" s="6" t="inlineStr">
         <is>
-          <t>713-2: AP World History - 2</t>
+          <t>711-2: World History H - 2</t>
         </is>
       </c>
       <c r="E723" s="6" t="inlineStr">
         <is>
-          <t>713-2: AP World History - 2</t>
+          <t>711-2: World History H - 2</t>
         </is>
       </c>
       <c r="F723" s="2" t="n"/>
@@ -20443,12 +20443,12 @@
       <c r="C724" s="2" t="n"/>
       <c r="D724" s="6" t="inlineStr">
         <is>
-          <t>711-2: World History H - 2</t>
+          <t>711-1: World History H - 1</t>
         </is>
       </c>
       <c r="E724" s="6" t="inlineStr">
         <is>
-          <t>711-2: World History H - 2</t>
+          <t>711-1: World History H - 1</t>
         </is>
       </c>
       <c r="F724" s="2" t="n"/>
@@ -20475,14 +20475,14 @@
         </is>
       </c>
       <c r="C725" s="2" t="n"/>
-      <c r="D725" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D725" s="6" t="inlineStr">
+        <is>
+          <t>713-2: AP World History - 2</t>
         </is>
       </c>
       <c r="E725" s="6" t="inlineStr">
         <is>
-          <t>744-2-S: Sociology - 2</t>
+          <t>713-2: AP World History - 2</t>
         </is>
       </c>
       <c r="F725" s="2" t="n"/>
@@ -20511,12 +20511,12 @@
       <c r="C726" s="2" t="n"/>
       <c r="D726" s="6" t="inlineStr">
         <is>
-          <t>711-1: World History H - 1</t>
+          <t>744-1-F: Sociology - 1</t>
         </is>
       </c>
       <c r="E726" s="6" t="inlineStr">
         <is>
-          <t>711-1: World History H - 1</t>
+          <t>744-2-S: Sociology - 2</t>
         </is>
       </c>
       <c r="F726" s="2" t="n"/>
@@ -20611,9 +20611,9 @@
         </is>
       </c>
       <c r="C729" s="2" t="n"/>
-      <c r="D729" s="6" t="inlineStr">
-        <is>
-          <t>744-1-F: Sociology - 1</t>
+      <c r="D729" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="E729" s="7" t="inlineStr">
@@ -20662,7 +20662,7 @@
       </c>
       <c r="C731" s="2" t="n"/>
       <c r="D731" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E731" s="9" t="n">
         <v>6</v>
@@ -21405,9 +21405,9 @@
           <t>751-1-F: American Government &amp; Politics - 1</t>
         </is>
       </c>
-      <c r="E759" s="6" t="inlineStr">
-        <is>
-          <t>741-2-S: Psychology - 2</t>
+      <c r="E759" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F759" s="2" t="n"/>
@@ -21468,14 +21468,14 @@
         </is>
       </c>
       <c r="C761" s="2" t="n"/>
-      <c r="D761" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E761" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D761" s="6" t="inlineStr">
+        <is>
+          <t>710-3: World History - 3</t>
+        </is>
+      </c>
+      <c r="E761" s="6" t="inlineStr">
+        <is>
+          <t>710-3: World History - 3</t>
         </is>
       </c>
       <c r="F761" s="2" t="n"/>
@@ -21504,12 +21504,12 @@
       <c r="C762" s="2" t="n"/>
       <c r="D762" s="6" t="inlineStr">
         <is>
-          <t>710-2: World History - 2</t>
-        </is>
-      </c>
-      <c r="E762" s="6" t="inlineStr">
-        <is>
-          <t>710-2: World History - 2</t>
+          <t>741-3-F: Psychology - 3</t>
+        </is>
+      </c>
+      <c r="E762" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F762" s="2" t="n"/>
@@ -21536,14 +21536,14 @@
         </is>
       </c>
       <c r="C763" s="2" t="n"/>
-      <c r="D763" s="6" t="inlineStr">
-        <is>
-          <t>741-3-F: Psychology - 3</t>
-        </is>
-      </c>
-      <c r="E763" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D763" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E763" s="6" t="inlineStr">
+        <is>
+          <t>741-2-S: Psychology - 2</t>
         </is>
       </c>
       <c r="F763" s="2" t="n"/>
@@ -21572,12 +21572,12 @@
       <c r="C764" s="2" t="n"/>
       <c r="D764" s="6" t="inlineStr">
         <is>
-          <t>710-3: World History - 3</t>
+          <t>710-2: World History - 2</t>
         </is>
       </c>
       <c r="E764" s="6" t="inlineStr">
         <is>
-          <t>710-3: World History - 3</t>
+          <t>710-2: World History - 2</t>
         </is>
       </c>
       <c r="F764" s="2" t="n"/>
@@ -21658,7 +21658,7 @@
         <v>4</v>
       </c>
       <c r="E767" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F767" s="2" t="n"/>
       <c r="G767" s="7" t="n">
@@ -21733,12 +21733,12 @@
       <c r="C771" s="2" t="n"/>
       <c r="D771" s="6" t="inlineStr">
         <is>
-          <t>110-5: Composition &amp; Literature - 5</t>
+          <t>110-4: Composition &amp; Literature - 4</t>
         </is>
       </c>
       <c r="E771" s="6" t="inlineStr">
         <is>
-          <t>110-5: Composition &amp; Literature - 5</t>
+          <t>110-4: Composition &amp; Literature - 4</t>
         </is>
       </c>
       <c r="F771" s="2" t="n"/>
@@ -21767,12 +21767,12 @@
       <c r="C772" s="2" t="n"/>
       <c r="D772" s="6" t="inlineStr">
         <is>
-          <t>110-4: Composition &amp; Literature - 4</t>
+          <t>110-5: Composition &amp; Literature - 5</t>
         </is>
       </c>
       <c r="E772" s="6" t="inlineStr">
         <is>
-          <t>110-4: Composition &amp; Literature - 4</t>
+          <t>110-5: Composition &amp; Literature - 5</t>
         </is>
       </c>
       <c r="F772" s="2" t="n"/>
@@ -21799,14 +21799,14 @@
         </is>
       </c>
       <c r="C773" s="2" t="n"/>
-      <c r="D773" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E773" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D773" s="6" t="inlineStr">
+        <is>
+          <t>110-2: Composition &amp; Literature - 2</t>
+        </is>
+      </c>
+      <c r="E773" s="6" t="inlineStr">
+        <is>
+          <t>110-2: Composition &amp; Literature - 2</t>
         </is>
       </c>
       <c r="F773" s="2" t="n"/>
@@ -21867,14 +21867,14 @@
         </is>
       </c>
       <c r="C775" s="2" t="n"/>
-      <c r="D775" s="6" t="inlineStr">
-        <is>
-          <t>110-2: Composition &amp; Literature - 2</t>
-        </is>
-      </c>
-      <c r="E775" s="6" t="inlineStr">
-        <is>
-          <t>110-2: Composition &amp; Literature - 2</t>
+      <c r="D775" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E775" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F775" s="2" t="n"/>
@@ -21985,11 +21985,11 @@
         </is>
       </c>
       <c r="C779" s="2" t="n"/>
-      <c r="D779" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E779" s="7" t="n">
-        <v>3</v>
+      <c r="D779" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E779" s="9" t="n">
+        <v>4</v>
       </c>
       <c r="F779" s="2" t="n"/>
       <c r="G779" s="9" t="n">
@@ -22461,14 +22461,14 @@
         </is>
       </c>
       <c r="C797" s="2" t="n"/>
-      <c r="D797" s="6" t="inlineStr">
-        <is>
-          <t>556-2: AP Physics - 2</t>
-        </is>
-      </c>
-      <c r="E797" s="6" t="inlineStr">
-        <is>
-          <t>556-2: AP Physics - 2</t>
+      <c r="D797" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E797" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F797" s="2" t="n"/>
@@ -22565,12 +22565,12 @@
       <c r="C800" s="2" t="n"/>
       <c r="D800" s="6" t="inlineStr">
         <is>
-          <t>556-1: AP Physics - 1</t>
+          <t>556-2: AP Physics - 2</t>
         </is>
       </c>
       <c r="E800" s="6" t="inlineStr">
         <is>
-          <t>556-1: AP Physics - 1</t>
+          <t>556-2: AP Physics - 2</t>
         </is>
       </c>
       <c r="F800" s="2" t="n"/>
@@ -22597,14 +22597,14 @@
         </is>
       </c>
       <c r="C801" s="2" t="n"/>
-      <c r="D801" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E801" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D801" s="6" t="inlineStr">
+        <is>
+          <t>556-1: AP Physics - 1</t>
+        </is>
+      </c>
+      <c r="E801" s="6" t="inlineStr">
+        <is>
+          <t>556-1: AP Physics - 1</t>
         </is>
       </c>
       <c r="F801" s="2" t="n"/>
@@ -22726,12 +22726,12 @@
       <c r="C807" s="2" t="n"/>
       <c r="D807" s="6" t="inlineStr">
         <is>
-          <t>310-5: Spanish I - 5</t>
+          <t>310-3: Spanish I - 3</t>
         </is>
       </c>
       <c r="E807" s="6" t="inlineStr">
         <is>
-          <t>310-5: Spanish I - 5</t>
+          <t>310-3: Spanish I - 3</t>
         </is>
       </c>
       <c r="F807" s="2" t="n"/>
@@ -22760,12 +22760,12 @@
       <c r="C808" s="2" t="n"/>
       <c r="D808" s="6" t="inlineStr">
         <is>
-          <t>310-4: Spanish I - 4</t>
+          <t>310-5: Spanish I - 5</t>
         </is>
       </c>
       <c r="E808" s="6" t="inlineStr">
         <is>
-          <t>310-4: Spanish I - 4</t>
+          <t>310-5: Spanish I - 5</t>
         </is>
       </c>
       <c r="F808" s="2" t="n"/>
@@ -22828,12 +22828,12 @@
       <c r="C810" s="2" t="n"/>
       <c r="D810" s="6" t="inlineStr">
         <is>
-          <t>310-3: Spanish I - 3</t>
+          <t>310-4: Spanish I - 4</t>
         </is>
       </c>
       <c r="E810" s="6" t="inlineStr">
         <is>
-          <t>310-3: Spanish I - 3</t>
+          <t>310-4: Spanish I - 4</t>
         </is>
       </c>
       <c r="F810" s="2" t="n"/>
@@ -22928,14 +22928,14 @@
         </is>
       </c>
       <c r="C813" s="2" t="n"/>
-      <c r="D813" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E813" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D813" s="6" t="inlineStr">
+        <is>
+          <t>310-6: Spanish I - 6</t>
+        </is>
+      </c>
+      <c r="E813" s="6" t="inlineStr">
+        <is>
+          <t>310-6: Spanish I - 6</t>
         </is>
       </c>
       <c r="F813" s="2" t="n"/>
@@ -22958,10 +22958,10 @@
       </c>
       <c r="C814" s="2" t="n"/>
       <c r="D814" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E814" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F814" s="2" t="n"/>
       <c r="G814" s="9" t="n">
@@ -23157,14 +23157,14 @@
         </is>
       </c>
       <c r="C822" s="2" t="n"/>
-      <c r="D822" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E822" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D822" s="6" t="inlineStr">
+        <is>
+          <t>130-5: British Literature - 5</t>
+        </is>
+      </c>
+      <c r="E822" s="6" t="inlineStr">
+        <is>
+          <t>130-5: British Literature - 5</t>
         </is>
       </c>
       <c r="F822" s="2" t="n"/>
@@ -23193,12 +23193,12 @@
       <c r="C823" s="2" t="n"/>
       <c r="D823" s="6" t="inlineStr">
         <is>
-          <t>130-4: British Literature - 4</t>
+          <t>130-3: British Literature - 3</t>
         </is>
       </c>
       <c r="E823" s="6" t="inlineStr">
         <is>
-          <t>130-4: British Literature - 4</t>
+          <t>130-3: British Literature - 3</t>
         </is>
       </c>
       <c r="F823" s="2" t="n"/>
@@ -23225,14 +23225,14 @@
         </is>
       </c>
       <c r="C824" s="2" t="n"/>
-      <c r="D824" s="6" t="inlineStr">
-        <is>
-          <t>130-5: British Literature - 5</t>
-        </is>
-      </c>
-      <c r="E824" s="6" t="inlineStr">
-        <is>
-          <t>130-5: British Literature - 5</t>
+      <c r="D824" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E824" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F824" s="2" t="n"/>
@@ -23261,12 +23261,12 @@
       <c r="C825" s="2" t="n"/>
       <c r="D825" s="6" t="inlineStr">
         <is>
-          <t>130-3: British Literature - 3</t>
+          <t>130-4: British Literature - 4</t>
         </is>
       </c>
       <c r="E825" s="6" t="inlineStr">
         <is>
-          <t>130-3: British Literature - 3</t>
+          <t>130-4: British Literature - 4</t>
         </is>
       </c>
       <c r="F825" s="2" t="n"/>
@@ -23309,11 +23309,11 @@
         </is>
       </c>
       <c r="C827" s="2" t="n"/>
-      <c r="D827" s="7" t="n">
-        <v>3</v>
+      <c r="D827" s="9" t="n">
+        <v>5</v>
       </c>
       <c r="E827" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F827" s="2" t="n"/>
       <c r="G827" s="7" t="n">
@@ -23785,14 +23785,14 @@
         </is>
       </c>
       <c r="C845" s="2" t="n"/>
-      <c r="D845" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E845" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D845" s="6" t="inlineStr">
+        <is>
+          <t>410-5: Algebra I - 5</t>
+        </is>
+      </c>
+      <c r="E845" s="6" t="inlineStr">
+        <is>
+          <t>410-5: Algebra I - 5</t>
         </is>
       </c>
       <c r="F845" s="2" t="n"/>
@@ -23819,14 +23819,14 @@
         </is>
       </c>
       <c r="C846" s="2" t="n"/>
-      <c r="D846" s="6" t="inlineStr">
-        <is>
-          <t>410-6: Algebra I - 6</t>
-        </is>
-      </c>
-      <c r="E846" s="6" t="inlineStr">
-        <is>
-          <t>410-6: Algebra I - 6</t>
+      <c r="D846" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E846" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F846" s="2" t="n"/>
@@ -23853,14 +23853,14 @@
         </is>
       </c>
       <c r="C847" s="2" t="n"/>
-      <c r="D847" s="6" t="inlineStr">
-        <is>
-          <t>410-5: Algebra I - 5</t>
-        </is>
-      </c>
-      <c r="E847" s="6" t="inlineStr">
-        <is>
-          <t>410-5: Algebra I - 5</t>
+      <c r="D847" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E847" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F847" s="2" t="n"/>
@@ -23921,14 +23921,14 @@
         </is>
       </c>
       <c r="C849" s="2" t="n"/>
-      <c r="D849" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E849" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D849" s="6" t="inlineStr">
+        <is>
+          <t>410-6: Algebra I - 6</t>
+        </is>
+      </c>
+      <c r="E849" s="6" t="inlineStr">
+        <is>
+          <t>410-6: Algebra I - 6</t>
         </is>
       </c>
       <c r="F849" s="2" t="n"/>
@@ -24150,14 +24150,14 @@
         </is>
       </c>
       <c r="C858" s="2" t="n"/>
-      <c r="D858" s="6" t="inlineStr">
-        <is>
-          <t>731-3: U.S. History II H - 3</t>
-        </is>
-      </c>
-      <c r="E858" s="6" t="inlineStr">
-        <is>
-          <t>731-3: U.S. History II H - 3</t>
+      <c r="D858" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E858" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F858" s="2" t="n"/>
@@ -24218,14 +24218,14 @@
         </is>
       </c>
       <c r="C860" s="2" t="n"/>
-      <c r="D860" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E860" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D860" s="6" t="inlineStr">
+        <is>
+          <t>710-6: World History - 6</t>
+        </is>
+      </c>
+      <c r="E860" s="6" t="inlineStr">
+        <is>
+          <t>710-6: World History - 6</t>
         </is>
       </c>
       <c r="F860" s="2" t="n"/>
@@ -24254,12 +24254,12 @@
       <c r="C861" s="2" t="n"/>
       <c r="D861" s="6" t="inlineStr">
         <is>
-          <t>710-6: World History - 6</t>
+          <t>731-3: U.S. History II H - 3</t>
         </is>
       </c>
       <c r="E861" s="6" t="inlineStr">
         <is>
-          <t>710-6: World History - 6</t>
+          <t>731-3: U.S. History II H - 3</t>
         </is>
       </c>
       <c r="F861" s="2" t="n"/>
@@ -24302,11 +24302,11 @@
         </is>
       </c>
       <c r="C863" s="2" t="n"/>
-      <c r="D863" s="9" t="n">
-        <v>5</v>
+      <c r="D863" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="E863" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F863" s="2" t="n"/>
       <c r="G863" s="9" t="n">
@@ -24483,12 +24483,12 @@
       <c r="C870" s="2" t="n"/>
       <c r="D870" s="6" t="inlineStr">
         <is>
-          <t>742-2: Economics - 2</t>
+          <t>742-1: Economics - 1</t>
         </is>
       </c>
       <c r="E870" s="6" t="inlineStr">
         <is>
-          <t>742-2: Economics - 2</t>
+          <t>742-1: Economics - 1</t>
         </is>
       </c>
       <c r="F870" s="2" t="n"/>
@@ -24517,12 +24517,12 @@
       <c r="C871" s="2" t="n"/>
       <c r="D871" s="6" t="inlineStr">
         <is>
-          <t>742-1: Economics - 1</t>
+          <t>742-2: Economics - 2</t>
         </is>
       </c>
       <c r="E871" s="6" t="inlineStr">
         <is>
-          <t>742-1: Economics - 1</t>
+          <t>742-2: Economics - 2</t>
         </is>
       </c>
       <c r="F871" s="2" t="n"/>
@@ -24710,14 +24710,14 @@
         </is>
       </c>
       <c r="C879" s="2" t="n"/>
-      <c r="D879" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
-        </is>
-      </c>
-      <c r="E879" s="7" t="inlineStr">
-        <is>
-          <t>UNASSIGNED</t>
+      <c r="D879" s="6" t="inlineStr">
+        <is>
+          <t>327-1: Latin II H - 1</t>
+        </is>
+      </c>
+      <c r="E879" s="6" t="inlineStr">
+        <is>
+          <t>327-1: Latin II H - 1</t>
         </is>
       </c>
       <c r="F879" s="2" t="n"/>
@@ -24914,14 +24914,14 @@
         </is>
       </c>
       <c r="C885" s="2" t="n"/>
-      <c r="D885" s="6" t="inlineStr">
-        <is>
-          <t>327-1: Latin II H - 1</t>
-        </is>
-      </c>
-      <c r="E885" s="6" t="inlineStr">
-        <is>
-          <t>327-1: Latin II H - 1</t>
+      <c r="D885" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
+        </is>
+      </c>
+      <c r="E885" s="7" t="inlineStr">
+        <is>
+          <t>UNASSIGNED</t>
         </is>
       </c>
       <c r="F885" s="2" t="n"/>

</xml_diff>